<commit_message>
fix crud and import data guru and siswa
</commit_message>
<xml_diff>
--- a/public/template_guru.xlsx
+++ b/public/template_guru.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SIMPEL-5\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53633061-7AE8-4E00-B79F-F96E92A89B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D18649-3907-4A88-8E7C-B8EC64F301EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9420" xr2:uid="{B5C1236F-2DC1-4DEB-9CB8-AC0626038A09}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B5C1236F-2DC1-4DEB-9CB8-AC0626038A09}"/>
   </bookViews>
   <sheets>
     <sheet name="Lembar1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>nama</t>
   </si>
@@ -42,28 +42,25 @@
     <t>program_studi</t>
   </si>
   <si>
-    <t>Manajemen Informatika</t>
-  </si>
-  <si>
-    <t>Teknologi Rekayasa Perangkat Lunak</t>
-  </si>
-  <si>
     <t>email</t>
   </si>
   <si>
     <t>nip</t>
   </si>
   <si>
-    <t>Nama Dosen 1</t>
-  </si>
-  <si>
-    <t>Nama Dosen 2</t>
-  </si>
-  <si>
-    <t>dosen1@gmail.com</t>
-  </si>
-  <si>
-    <t>dosen2@gmail.com</t>
+    <t>Multimedia</t>
+  </si>
+  <si>
+    <t>dosen5@gmail.com</t>
+  </si>
+  <si>
+    <t>dosen6@gmail.com</t>
+  </si>
+  <si>
+    <t>Guru 5</t>
+  </si>
+  <si>
+    <t>Guru 6</t>
   </si>
 </sst>
 </file>
@@ -134,7 +131,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hipertaut" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -151,7 +148,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -448,55 +445,55 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFAD8768-4066-4A27-B449-170C24190DD5}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.5546875" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" customWidth="1"/>
-    <col min="3" max="3" width="38.44140625" customWidth="1"/>
-    <col min="4" max="4" width="27.6640625" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="1" max="1" width="24.54296875" customWidth="1"/>
+    <col min="2" max="2" width="17.90625" customWidth="1"/>
+    <col min="3" max="3" width="38.453125" customWidth="1"/>
+    <col min="4" max="4" width="27.6328125" customWidth="1"/>
+    <col min="5" max="5" width="8.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2">
         <v>1920239852</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
       </c>
       <c r="B3" s="2">
         <v>1920239876</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>